<commit_message>
chore: update Instagram report 2026-08-31 05:53
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/2026-08-31.xlsx
+++ b/instagram-daily-checker/reports/2026-08-31.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-08-31 00:58:56</t>
+          <t>取得日時：2026-08-31 05:53:09</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1533</t>
+          <t>1534</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1568,12 +1568,12 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>161</t>
+          <t>162</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>+2人</t>
+          <t>+3人</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">

</xml_diff>